<commit_message>
Atualiza notas 3E Manha 2º Bimestre
</commit_message>
<xml_diff>
--- a/sources/3E_Manha_2_Bimestre.xlsx
+++ b/sources/3E_Manha_2_Bimestre.xlsx
@@ -61,7 +61,7 @@
     <x:t>Conselho Segundo Bimestre</x:t>
   </x:si>
   <x:si>
-    <x:t>245</x:t>
+    <x:t>320</x:t>
   </x:si>
   <x:si>
     <x:t>0 (Soma de todas as eletivas)</x:t>
@@ -222,240 +222,246 @@
     <x:t>17</x:t>
   </x:si>
   <x:si>
+    <x:t>24</x:t>
+  </x:si>
+  <x:si>
     <x:t>1</x:t>
   </x:si>
   <x:si>
     <x:t>16</x:t>
   </x:si>
   <x:si>
+    <x:t>58%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>67%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANA BEATRIZ CAVALCANTI MATOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>11</x:t>
+  </x:si>
+  <x:si>
+    <x:t>12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>72%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>78%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ANNA LAURA DOS SANTOS ALVES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>79%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>84%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DOMINGOS VICTOR LUZOLO JOAO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Não Comparecimento</x:t>
+  </x:si>
+  <x:si>
+    <x:t>100%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>EMANUELLY LORRAINE DE ASSIS DE OLIVEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>22</x:t>
+  </x:si>
+  <x:si>
+    <x:t>65%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>56%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FELIPI GUSTAVO PAQUIELA DE OLIVEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>83%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>FERNANDO MEDEIROS DA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>89%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>87%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GABRIEL OLIVEIRA GONÇALVES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Baixa - Transferência</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GABRIEL STEVANIN TAVARES JULIANO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GERTUDES ZAU MBUANGI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>88%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GRAZIELLE BARROS DE MEDEIROS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUILHERME ALVES VIEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>86%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUILHERME DOS SANTOS ARANTES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>77%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUILHERME SILVA DE PAULA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>80%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GUSTAVO CAETANO SOLOVIOW DE OLIVEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>85%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HALANNA DE ALMEIDA OLTRAMARI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>13</x:t>
+  </x:si>
+  <x:si>
+    <x:t>82%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HENRY OLIVEIRA DE FRANÇA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>93%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>95%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IGOR CASTILHO PARAVANI DE SOUZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>90%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ISABELLA ARCHAPA NASCIMENTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>JOSE XAVIER ALVES FILHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>98%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>99%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>KAUAN DOS SANTOS MELO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LETHICIA DOS SANTOS BORTUNI</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUCAS EVANGELISTA DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>68%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>69%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>LUIZ GUSTAVO MARIANO DO NASCIMENTO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARCUS VINICIUS DA COSTA SILVA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>30</x:t>
+  </x:si>
+  <x:si>
+    <x:t>55%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>52%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARIA EDUARDA RITA BATISTA VIEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MARIANA ESTEFANI FERREIRA MIRANDA</x:t>
+  </x:si>
+  <x:si>
     <x:t>60%</x:t>
   </x:si>
   <x:si>
-    <x:t>68%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANA BEATRIZ CAVALCANTI MATOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>11</x:t>
-  </x:si>
-  <x:si>
-    <x:t>12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>71%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>79%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ANNA LAURA DOS SANTOS ALVES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>85%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DOMINGOS VICTOR LUZOLO JOAO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Não Comparecimento</x:t>
-  </x:si>
-  <x:si>
-    <x:t>100%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>EMANUELLY LORRAINE DE ASSIS DE OLIVEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>22</x:t>
-  </x:si>
-  <x:si>
-    <x:t>55%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>50%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FELIPI GUSTAVO PAQUIELA DE OLIVEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>80%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>84%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>FERNANDO MEDEIROS DA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>90%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>87%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GABRIEL OLIVEIRA GONÇALVES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Baixa - Transferência</x:t>
+    <x:t>MATHEUS ARTHUR FROTA DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>81%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>MOISES BATISTA VIEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NICOLE NOGUEIRA DAMIAO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>91%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>PABLO KILDEY DA SILVA RAMALHO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Remanejamento</x:t>
   </x:si>
   <x:si>
     <x:t>76%</x:t>
   </x:si>
   <x:si>
-    <x:t>GABRIEL STEVANIN TAVARES JULIANO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>86%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GERTUDES ZAU MBUANGI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GRAZIELLE BARROS DE MEDEIROS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>88%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUILHERME ALVES VIEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUILHERME DOS SANTOS ARANTES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>77%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUILHERME SILVA DE PAULA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GUSTAVO CAETANO SOLOVIOW DE OLIVEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>82%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HALANNA DE ALMEIDA OLTRAMARI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>78%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HENRY OLIVEIRA DE FRANÇA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>93%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>95%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>IGOR CASTILHO PARAVANI DE SOUZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>91%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ISABELLA ARCHAPA NASCIMENTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>JOSE XAVIER ALVES FILHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>98%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>99%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>KAUAN DOS SANTOS MELO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LETHICIA DOS SANTOS BORTUNI</x:t>
-  </x:si>
-  <x:si>
-    <x:t>89%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LUCAS EVANGELISTA DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>69%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>LUIZ GUSTAVO MARIANO DO NASCIMENTO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARCUS VINICIUS DA COSTA SILVA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>20</x:t>
-  </x:si>
-  <x:si>
-    <x:t>30</x:t>
-  </x:si>
-  <x:si>
-    <x:t>41%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>45%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARIA EDUARDA RITA BATISTA VIEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>83%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MARIANA ESTEFANI FERREIRA MIRANDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>72%</x:t>
+    <x:t>PAULO RICARDO PEREIRA LOPES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>THAÍNA LEMES DE OLIVEIRA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RAQUEL POTENCIANA SANDA MPATA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RUAN ANDRADE DOS SANTOS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>26</x:t>
   </x:si>
   <x:si>
     <x:t>54%</x:t>
   </x:si>
   <x:si>
-    <x:t>MATHEUS ARTHUR FROTA DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>MOISES BATISTA VIEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NICOLE NOGUEIRA DAMIAO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PABLO KILDEY DA SILVA RAMALHO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Remanejamento</x:t>
-  </x:si>
-  <x:si>
-    <x:t>73%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>PAULO RICARDO PEREIRA LOPES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>THAÍNA LEMES DE OLIVEIRA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RAQUEL POTENCIANA SANDA MPATA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RUAN ANDRADE DOS SANTOS</x:t>
-  </x:si>
-  <x:si>
-    <x:t>26</x:t>
-  </x:si>
-  <x:si>
-    <x:t>42%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>47%</x:t>
-  </x:si>
-  <x:si>
     <x:t>RYAN SOARES AQUINO</x:t>
   </x:si>
   <x:si>
@@ -465,42 +471,33 @@
     <x:t>VICTOR HIROSHI ASSAKAWA KASAMATU</x:t>
   </x:si>
   <x:si>
-    <x:t>81%</x:t>
+    <x:t>VINICIUS GIMENEZ DA COSTA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>WENDEL RAMOS DELFINO DE SOUZA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>63%</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ZION KALUEMBI SANTOS PORTELA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>YUMI EUGENIO URATA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RYAN GUEDES DE BRITO FRANCISCO</x:t>
+  </x:si>
+  <x:si>
+    <x:t>NICOLAS MARCON MARQUES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>DANIELA RAMOS MIRANDA</x:t>
   </x:si>
   <x:si>
     <x:t>75%</x:t>
   </x:si>
   <x:si>
-    <x:t>VINICIUS GIMENEZ DA COSTA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>WENDEL RAMOS DELFINO DE SOUZA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>15</x:t>
-  </x:si>
-  <x:si>
-    <x:t>64%</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ZION KALUEMBI SANTOS PORTELA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>YUMI EUGENIO URATA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RYAN GUEDES DE BRITO FRANCISCO</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NICOLAS MARCON MARQUES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>DANIELA RAMOS MIRANDA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>74%</x:t>
-  </x:si>
-  <x:si>
     <x:t>ELOISE DE CARVALHO GONCALVES</x:t>
   </x:si>
   <x:si>
@@ -531,7 +528,13 @@
     <x:t>Aulas Dadas: 48</x:t>
   </x:si>
   <x:si>
+    <x:t>Aulas Dadas: 50</x:t>
+  </x:si>
+  <x:si>
     <x:t>Aulas Dadas: 34</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Aulas Dadas: 25</x:t>
   </x:si>
   <x:si>
     <x:t>Aulas Dadas: 10</x:t>
@@ -1572,13 +1575,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AJ13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM13" s="12">
         <x:v>1</x:v>
@@ -1596,13 +1599,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="AR13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AS13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT13" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU13" s="12">
         <x:v>1</x:v>
@@ -1641,13 +1644,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG13" s="12">
-        <x:v>20</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="BH13" s="12" t="s">
         <x:v>56</x:v>
       </x:c>
       <x:c r="BI13" s="12">
-        <x:v>33</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="BJ13" s="12" t="s">
         <x:v>57</x:v>
@@ -1760,13 +1763,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AJ14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="AL14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM14" s="12">
         <x:v>2</x:v>
@@ -1784,19 +1787,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="AR14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AT14" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU14" s="12">
         <x:v>2</x:v>
       </x:c>
       <x:c r="AV14" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AW14" s="12" t="s">
         <x:v>48</x:v>
@@ -1823,27 +1826,27 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="BE14" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="BF14" s="12" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG14" s="12">
-        <x:v>99</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="BH14" s="12" t="s">
-        <x:v>66</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="BI14" s="12">
-        <x:v>180</x:v>
+        <x:v>214</x:v>
       </x:c>
       <x:c r="BJ14" s="12" t="s">
-        <x:v>67</x:v>
+        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:62">
       <x:c r="A15" s="11" t="s">
-        <x:v>68</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B15" s="12" t="s">
         <x:v>47</x:v>
@@ -1927,7 +1930,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="AC15" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="AD15" s="12" t="s">
         <x:v>48</x:v>
@@ -1939,7 +1942,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="AG15" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AH15" s="12" t="s">
         <x:v>49</x:v>
@@ -1948,13 +1951,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="AJ15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="AL15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM15" s="12">
         <x:v>3</x:v>
@@ -1972,13 +1975,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="AR15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT15" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU15" s="12">
         <x:v>3</x:v>
@@ -1999,7 +2002,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BA15" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB15" s="12" t="s">
         <x:v>49</x:v>
@@ -2011,27 +2014,27 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="BE15" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="BF15" s="12" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG15" s="12">
-        <x:v>71</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="BH15" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BI15" s="12">
-        <x:v>121</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="BJ15" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:62">
       <x:c r="A16" s="11" t="s">
-        <x:v>73</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="B16" s="12" t="s">
         <x:v>47</x:v>
@@ -2094,7 +2097,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="V16" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="W16" s="12">
         <x:v>4</x:v>
@@ -2136,13 +2139,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AJ16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="AL16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM16" s="12">
         <x:v>4</x:v>
@@ -2160,13 +2163,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="AR16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AS16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT16" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU16" s="12">
         <x:v>4</x:v>
@@ -2199,30 +2202,30 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="BE16" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="BF16" s="12" t="s">
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG16" s="12">
-        <x:v>51</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="BH16" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="BI16" s="12">
-        <x:v>84</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BJ16" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:62">
       <x:c r="A17" s="11" t="s">
-        <x:v>75</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B17" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C17" s="12">
         <x:v>5</x:v>
@@ -2327,10 +2330,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK17" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL17" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM17" s="12">
         <x:v>5</x:v>
@@ -2351,10 +2354,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS17" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT17" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU17" s="12">
         <x:v>5</x:v>
@@ -2396,21 +2399,21 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH17" s="12" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BI17" s="12">
         <x:v>171</x:v>
       </x:c>
       <x:c r="BJ17" s="12" t="s">
-        <x:v>67</x:v>
+        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:62">
       <x:c r="A18" s="11" t="s">
+        <x:v>80</x:v>
+      </x:c>
+      <x:c r="B18" s="12" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="B18" s="12" t="s">
-        <x:v>76</x:v>
       </x:c>
       <x:c r="C18" s="12">
         <x:v>6</x:v>
@@ -2503,7 +2506,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AG18" s="12" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="AH18" s="12" t="s">
         <x:v>49</x:v>
@@ -2515,10 +2518,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK18" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL18" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM18" s="12">
         <x:v>6</x:v>
@@ -2527,7 +2530,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO18" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AP18" s="12" t="s">
         <x:v>49</x:v>
@@ -2539,10 +2542,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS18" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT18" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU18" s="12">
         <x:v>6</x:v>
@@ -2575,7 +2578,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BE18" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="BF18" s="12" t="s">
         <x:v>49</x:v>
@@ -2584,18 +2587,18 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="BH18" s="12" t="s">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="BI18" s="12">
         <x:v>269</x:v>
       </x:c>
       <x:c r="BJ18" s="12" t="s">
-        <x:v>81</x:v>
+        <x:v>83</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:62">
       <x:c r="A19" s="11" t="s">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="B19" s="12" t="s">
         <x:v>47</x:v>
@@ -2700,13 +2703,13 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="AJ19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AL19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM19" s="12">
         <x:v>7</x:v>
@@ -2724,13 +2727,13 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="AR19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT19" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU19" s="12">
         <x:v>7</x:v>
@@ -2769,21 +2772,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG19" s="12">
-        <x:v>49</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="BH19" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="BI19" s="12">
-        <x:v>89</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="BJ19" s="12" t="s">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:62">
       <x:c r="A20" s="11" t="s">
-        <x:v>85</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B20" s="12" t="s">
         <x:v>47</x:v>
@@ -2888,13 +2891,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="AJ20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AL20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM20" s="12">
         <x:v>8</x:v>
@@ -2912,13 +2915,13 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="AR20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AS20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT20" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU20" s="12">
         <x:v>8</x:v>
@@ -2939,7 +2942,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="BA20" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB20" s="12" t="s">
         <x:v>49</x:v>
@@ -2957,24 +2960,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG20" s="12">
-        <x:v>25</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="BH20" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BI20" s="12">
-        <x:v>74</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="BJ20" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:62">
       <x:c r="A21" s="11" t="s">
-        <x:v>88</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B21" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C21" s="12">
         <x:v>9</x:v>
@@ -3007,7 +3010,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="M21" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N21" s="12" t="s">
         <x:v>49</x:v>
@@ -3079,10 +3082,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK21" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL21" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM21" s="12">
         <x:v>9</x:v>
@@ -3103,10 +3106,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS21" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT21" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU21" s="12">
         <x:v>9</x:v>
@@ -3127,7 +3130,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="BA21" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB21" s="12" t="s">
         <x:v>49</x:v>
@@ -3148,13 +3151,13 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="BH21" s="12" t="s">
-        <x:v>56</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="BI21" s="12">
         <x:v>131</x:v>
       </x:c>
       <x:c r="BJ21" s="12" t="s">
-        <x:v>90</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:62">
@@ -3264,13 +3267,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="AJ22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="AL22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM22" s="12">
         <x:v>10</x:v>
@@ -3288,13 +3291,13 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="AR22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT22" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU22" s="12">
         <x:v>10</x:v>
@@ -3315,7 +3318,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="BA22" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB22" s="12" t="s">
         <x:v>49</x:v>
@@ -3333,21 +3336,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG22" s="12">
-        <x:v>35</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="BH22" s="12" t="s">
-        <x:v>92</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="BI22" s="12">
-        <x:v>58</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="BJ22" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:62">
       <x:c r="A23" s="11" t="s">
-        <x:v>93</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B23" s="12" t="s">
         <x:v>47</x:v>
@@ -3383,7 +3386,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="M23" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N23" s="12" t="s">
         <x:v>49</x:v>
@@ -3452,13 +3455,13 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="AJ23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM23" s="12">
         <x:v>11</x:v>
@@ -3476,13 +3479,13 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="AR23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT23" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU23" s="12">
         <x:v>11</x:v>
@@ -3503,7 +3506,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="BA23" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB23" s="12" t="s">
         <x:v>49</x:v>
@@ -3521,16 +3524,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG23" s="12">
-        <x:v>34</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="BH23" s="12" t="s">
-        <x:v>92</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="BI23" s="12">
-        <x:v>71</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="BJ23" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:62">
@@ -3571,7 +3574,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="M24" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N24" s="12" t="s">
         <x:v>49</x:v>
@@ -3640,13 +3643,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="AJ24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AK24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="AL24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM24" s="12">
         <x:v>12</x:v>
@@ -3664,13 +3667,13 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="AR24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AS24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT24" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU24" s="12">
         <x:v>12</x:v>
@@ -3709,16 +3712,16 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG24" s="12">
-        <x:v>50</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="BH24" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="BI24" s="12">
-        <x:v>68</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="BJ24" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:62">
@@ -3828,13 +3831,13 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="AJ25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AL25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM25" s="12">
         <x:v>13</x:v>
@@ -3852,13 +3855,13 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="AR25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT25" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU25" s="12">
         <x:v>13</x:v>
@@ -3897,21 +3900,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG25" s="12">
-        <x:v>36</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="BH25" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI25" s="12">
-        <x:v>73</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="BJ25" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:62">
       <x:c r="A26" s="11" t="s">
-        <x:v>97</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="B26" s="12" t="s">
         <x:v>47</x:v>
@@ -3947,7 +3950,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="M26" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N26" s="12" t="s">
         <x:v>49</x:v>
@@ -4016,13 +4019,13 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="AJ26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AL26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM26" s="12">
         <x:v>14</x:v>
@@ -4040,13 +4043,13 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="AR26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT26" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU26" s="12">
         <x:v>14</x:v>
@@ -4085,21 +4088,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG26" s="12">
-        <x:v>57</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="BH26" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="BI26" s="12">
-        <x:v>121</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="BJ26" s="12" t="s">
-        <x:v>72</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:62">
       <x:c r="A27" s="11" t="s">
-        <x:v>99</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B27" s="12" t="s">
         <x:v>47</x:v>
@@ -4183,7 +4186,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="AC27" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="AD27" s="12" t="s">
         <x:v>61</x:v>
@@ -4195,7 +4198,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="AG27" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AH27" s="12" t="s">
         <x:v>49</x:v>
@@ -4204,13 +4207,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="AJ27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AL27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM27" s="12">
         <x:v>15</x:v>
@@ -4228,13 +4231,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="AR27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT27" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU27" s="12">
         <x:v>15</x:v>
@@ -4255,7 +4258,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="BA27" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB27" s="12" t="s">
         <x:v>49</x:v>
@@ -4273,21 +4276,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG27" s="12">
-        <x:v>60</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BH27" s="12" t="s">
-        <x:v>90</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="BI27" s="12">
-        <x:v>114</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="BJ27" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>101</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:62">
       <x:c r="A28" s="11" t="s">
-        <x:v>100</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="B28" s="12" t="s">
         <x:v>47</x:v>
@@ -4392,13 +4395,13 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="AJ28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AL28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM28" s="12">
         <x:v>16</x:v>
@@ -4416,13 +4419,13 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="AR28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT28" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU28" s="12">
         <x:v>16</x:v>
@@ -4443,7 +4446,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="BA28" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB28" s="12" t="s">
         <x:v>49</x:v>
@@ -4461,21 +4464,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG28" s="12">
-        <x:v>45</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="BH28" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="BI28" s="12">
-        <x:v>89</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="BJ28" s="12" t="s">
-        <x:v>84</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:62">
       <x:c r="A29" s="11" t="s">
-        <x:v>102</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="B29" s="12" t="s">
         <x:v>47</x:v>
@@ -4580,13 +4583,13 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="AJ29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="AL29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM29" s="12">
         <x:v>17</x:v>
@@ -4604,13 +4607,13 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="AR29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AS29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT29" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU29" s="12">
         <x:v>17</x:v>
@@ -4649,21 +4652,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG29" s="12">
-        <x:v>54</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="BH29" s="12" t="s">
-        <x:v>103</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="BI29" s="12">
-        <x:v>101</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="BJ29" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:62">
       <x:c r="A30" s="11" t="s">
-        <x:v>104</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B30" s="12" t="s">
         <x:v>47</x:v>
@@ -4699,7 +4702,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="M30" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N30" s="12" t="s">
         <x:v>49</x:v>
@@ -4768,13 +4771,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="AJ30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AL30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM30" s="12">
         <x:v>18</x:v>
@@ -4792,13 +4795,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="AR30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT30" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU30" s="12">
         <x:v>18</x:v>
@@ -4837,21 +4840,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG30" s="12">
-        <x:v>17</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="BH30" s="12" t="s">
-        <x:v>105</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="BI30" s="12">
-        <x:v>26</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="BJ30" s="12" t="s">
-        <x:v>106</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:62">
       <x:c r="A31" s="11" t="s">
-        <x:v>107</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B31" s="12" t="s">
         <x:v>47</x:v>
@@ -4887,7 +4890,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="M31" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N31" s="12" t="s">
         <x:v>49</x:v>
@@ -4956,13 +4959,13 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="AJ31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AL31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM31" s="12">
         <x:v>19</x:v>
@@ -4980,13 +4983,13 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="AR31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT31" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU31" s="12">
         <x:v>19</x:v>
@@ -5025,21 +5028,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG31" s="12">
-        <x:v>37</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="BH31" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="BI31" s="12">
-        <x:v>52</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="BJ31" s="12" t="s">
-        <x:v>108</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:62">
       <x:c r="A32" s="11" t="s">
-        <x:v>109</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B32" s="12" t="s">
         <x:v>47</x:v>
@@ -5075,7 +5078,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="M32" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N32" s="12" t="s">
         <x:v>49</x:v>
@@ -5144,13 +5147,13 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="AJ32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AL32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM32" s="12">
         <x:v>20</x:v>
@@ -5168,19 +5171,19 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="AR32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AS32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT32" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU32" s="12">
         <x:v>20</x:v>
       </x:c>
       <x:c r="AV32" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AW32" s="12" t="s">
         <x:v>54</x:v>
@@ -5213,21 +5216,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG32" s="12">
-        <x:v>45</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="BH32" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BI32" s="12">
-        <x:v>50</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="BJ32" s="12" t="s">
-        <x:v>108</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="33" spans="1:62">
       <x:c r="A33" s="11" t="s">
-        <x:v>110</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B33" s="12" t="s">
         <x:v>47</x:v>
@@ -5263,10 +5266,10 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="M33" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N33" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="O33" s="12">
         <x:v>21</x:v>
@@ -5332,13 +5335,13 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="AJ33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM33" s="12">
         <x:v>21</x:v>
@@ -5356,13 +5359,13 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="AR33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT33" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU33" s="12">
         <x:v>21</x:v>
@@ -5383,10 +5386,10 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="BA33" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB33" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BC33" s="12">
         <x:v>21</x:v>
@@ -5401,21 +5404,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG33" s="12">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="BH33" s="12" t="s">
-        <x:v>111</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="BI33" s="12">
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="BJ33" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:62">
       <x:c r="A34" s="11" t="s">
-        <x:v>113</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B34" s="12" t="s">
         <x:v>47</x:v>
@@ -5520,13 +5523,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="AJ34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM34" s="12">
         <x:v>22</x:v>
@@ -5544,13 +5547,13 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="AR34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AS34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT34" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU34" s="12">
         <x:v>22</x:v>
@@ -5589,21 +5592,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG34" s="12">
-        <x:v>34</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="BH34" s="12" t="s">
+        <x:v>88</x:v>
+      </x:c>
+      <x:c r="BI34" s="12">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="BI34" s="12">
-        <x:v>84</x:v>
-      </x:c>
       <x:c r="BJ34" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="35" spans="1:62">
       <x:c r="A35" s="11" t="s">
-        <x:v>114</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B35" s="12" t="s">
         <x:v>47</x:v>
@@ -5708,13 +5711,13 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="AJ35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM35" s="12">
         <x:v>23</x:v>
@@ -5732,13 +5735,13 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="AR35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AS35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AT35" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU35" s="12">
         <x:v>23</x:v>
@@ -5777,21 +5780,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG35" s="12">
-        <x:v>30</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="BH35" s="12" t="s">
-        <x:v>95</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="BI35" s="12">
-        <x:v>60</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BJ35" s="12" t="s">
-        <x:v>115</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="36" spans="1:62">
       <x:c r="A36" s="11" t="s">
-        <x:v>116</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="B36" s="12" t="s">
         <x:v>47</x:v>
@@ -5872,10 +5875,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="AB36" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AC36" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="AD36" s="12" t="s">
         <x:v>48</x:v>
@@ -5896,13 +5899,13 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="AJ36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AK36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="AL36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM36" s="12">
         <x:v>24</x:v>
@@ -5920,13 +5923,13 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="AR36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AS36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AT36" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU36" s="12">
         <x:v>24</x:v>
@@ -5965,21 +5968,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG36" s="12">
-        <x:v>78</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BH36" s="12" t="s">
-        <x:v>67</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="BI36" s="12">
-        <x:v>177</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="BJ36" s="12" t="s">
-        <x:v>117</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="37" spans="1:62">
       <x:c r="A37" s="11" t="s">
-        <x:v>118</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B37" s="12" t="s">
         <x:v>47</x:v>
@@ -6084,13 +6087,13 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="AJ37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="AL37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM37" s="12">
         <x:v>25</x:v>
@@ -6108,13 +6111,13 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="AR37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT37" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU37" s="12">
         <x:v>25</x:v>
@@ -6153,24 +6156,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG37" s="12">
-        <x:v>44</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="BH37" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BI37" s="12">
-        <x:v>49</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="BJ37" s="12" t="s">
-        <x:v>108</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="38" spans="1:62">
       <x:c r="A38" s="11" t="s">
-        <x:v>119</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B38" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C38" s="12">
         <x:v>26</x:v>
@@ -6191,7 +6194,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="I38" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="J38" s="12" t="s">
         <x:v>49</x:v>
@@ -6248,10 +6251,10 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="AB38" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AC38" s="12" t="s">
-        <x:v>120</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="AD38" s="12" t="s">
         <x:v>49</x:v>
@@ -6263,7 +6266,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AG38" s="12" t="s">
-        <x:v>121</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="AH38" s="12" t="s">
         <x:v>49</x:v>
@@ -6275,10 +6278,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK38" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL38" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM38" s="12">
         <x:v>26</x:v>
@@ -6287,7 +6290,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO38" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AP38" s="12" t="s">
         <x:v>49</x:v>
@@ -6299,10 +6302,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS38" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT38" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU38" s="12">
         <x:v>26</x:v>
@@ -6335,7 +6338,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BE38" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="BF38" s="12" t="s">
         <x:v>49</x:v>
@@ -6344,18 +6347,18 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="BH38" s="12" t="s">
-        <x:v>122</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="BI38" s="12">
         <x:v>298</x:v>
       </x:c>
       <x:c r="BJ38" s="12" t="s">
-        <x:v>123</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="39" spans="1:62">
       <x:c r="A39" s="11" t="s">
-        <x:v>124</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B39" s="12" t="s">
         <x:v>47</x:v>
@@ -6391,7 +6394,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="M39" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N39" s="12" t="s">
         <x:v>49</x:v>
@@ -6460,13 +6463,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="AJ39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AL39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM39" s="12">
         <x:v>27</x:v>
@@ -6484,13 +6487,13 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="AR39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT39" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU39" s="12">
         <x:v>27</x:v>
@@ -6511,7 +6514,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="BA39" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB39" s="12" t="s">
         <x:v>49</x:v>
@@ -6529,24 +6532,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG39" s="12">
-        <x:v>44</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="BH39" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BI39" s="12">
-        <x:v>94</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="BJ39" s="12" t="s">
-        <x:v>125</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="40" spans="1:62">
       <x:c r="A40" s="11" t="s">
-        <x:v>126</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="B40" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C40" s="12">
         <x:v>28</x:v>
@@ -6651,10 +6654,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK40" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL40" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM40" s="12">
         <x:v>28</x:v>
@@ -6675,10 +6678,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS40" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT40" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU40" s="12">
         <x:v>28</x:v>
@@ -6720,18 +6723,18 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="BH40" s="12" t="s">
-        <x:v>127</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="BI40" s="12">
         <x:v>247</x:v>
       </x:c>
       <x:c r="BJ40" s="12" t="s">
-        <x:v>128</x:v>
+        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="41" spans="1:62">
       <x:c r="A41" s="11" t="s">
-        <x:v>129</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B41" s="12" t="s">
         <x:v>47</x:v>
@@ -6794,7 +6797,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="V41" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="W41" s="12">
         <x:v>29</x:v>
@@ -6836,13 +6839,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="AJ41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AL41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM41" s="12">
         <x:v>29</x:v>
@@ -6860,13 +6863,13 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="AR41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT41" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU41" s="12">
         <x:v>29</x:v>
@@ -6905,21 +6908,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG41" s="12">
-        <x:v>43</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="BH41" s="12" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="BI41" s="12">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="BI41" s="12">
-        <x:v>83</x:v>
-      </x:c>
       <x:c r="BJ41" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
     </x:row>
     <x:row r="42" spans="1:62">
       <x:c r="A42" s="11" t="s">
-        <x:v>130</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="B42" s="12" t="s">
         <x:v>47</x:v>
@@ -7015,7 +7018,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="AG42" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AH42" s="12" t="s">
         <x:v>49</x:v>
@@ -7024,13 +7027,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="AJ42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AL42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM42" s="12">
         <x:v>30</x:v>
@@ -7048,13 +7051,13 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="AR42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AT42" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU42" s="12">
         <x:v>30</x:v>
@@ -7093,21 +7096,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG42" s="12">
-        <x:v>48</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="BH42" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="BI42" s="12">
-        <x:v>90</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BJ42" s="12" t="s">
-        <x:v>84</x:v>
+        <x:v>85</x:v>
       </x:c>
     </x:row>
     <x:row r="43" spans="1:62">
       <x:c r="A43" s="11" t="s">
-        <x:v>131</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B43" s="12" t="s">
         <x:v>47</x:v>
@@ -7212,13 +7215,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="AJ43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AL43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM43" s="12">
         <x:v>31</x:v>
@@ -7236,13 +7239,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="AR43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT43" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU43" s="12">
         <x:v>31</x:v>
@@ -7281,24 +7284,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG43" s="12">
-        <x:v>36</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="BH43" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="BI43" s="12">
-        <x:v>51</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="BJ43" s="12" t="s">
-        <x:v>108</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:62">
       <x:c r="A44" s="11" t="s">
-        <x:v>132</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B44" s="12" t="s">
-        <x:v>133</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C44" s="12">
         <x:v>32</x:v>
@@ -7403,10 +7406,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK44" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL44" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM44" s="12">
         <x:v>32</x:v>
@@ -7427,10 +7430,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS44" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT44" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU44" s="12">
         <x:v>32</x:v>
@@ -7472,18 +7475,18 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="BH44" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="BI44" s="12">
         <x:v>148</x:v>
       </x:c>
       <x:c r="BJ44" s="12" t="s">
-        <x:v>134</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:62">
       <x:c r="A45" s="11" t="s">
-        <x:v>135</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B45" s="12" t="s">
         <x:v>47</x:v>
@@ -7588,13 +7591,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AJ45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AL45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM45" s="12">
         <x:v>33</x:v>
@@ -7612,13 +7615,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="AR45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AS45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT45" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU45" s="12">
         <x:v>33</x:v>
@@ -7657,21 +7660,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG45" s="12">
-        <x:v>38</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="BH45" s="12" t="s">
-        <x:v>84</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="BI45" s="12">
-        <x:v>57</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="BJ45" s="12" t="s">
-        <x:v>86</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="46" spans="1:62">
       <x:c r="A46" s="11" t="s">
-        <x:v>136</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B46" s="12" t="s">
         <x:v>47</x:v>
@@ -7707,7 +7710,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="M46" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N46" s="12" t="s">
         <x:v>49</x:v>
@@ -7734,7 +7737,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="V46" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="W46" s="12">
         <x:v>34</x:v>
@@ -7776,13 +7779,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="AJ46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AL46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM46" s="12">
         <x:v>34</x:v>
@@ -7800,13 +7803,13 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="AR46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT46" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU46" s="12">
         <x:v>34</x:v>
@@ -7827,7 +7830,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="BA46" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB46" s="12" t="s">
         <x:v>49</x:v>
@@ -7845,21 +7848,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG46" s="12">
-        <x:v>50</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="BH46" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="BI46" s="12">
-        <x:v>127</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="BJ46" s="12" t="s">
-        <x:v>98</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="47" spans="1:62">
       <x:c r="A47" s="11" t="s">
-        <x:v>137</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="B47" s="12" t="s">
         <x:v>47</x:v>
@@ -7964,13 +7967,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="AJ47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM47" s="12">
         <x:v>35</x:v>
@@ -7988,13 +7991,13 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="AR47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AT47" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU47" s="12">
         <x:v>35</x:v>
@@ -8033,24 +8036,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG47" s="12">
-        <x:v>36</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="BH47" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="BI47" s="12">
-        <x:v>87</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="BJ47" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="48" spans="1:62">
       <x:c r="A48" s="11" t="s">
-        <x:v>138</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B48" s="12" t="s">
-        <x:v>76</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C48" s="12">
         <x:v>36</x:v>
@@ -8080,7 +8083,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="L48" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="M48" s="12" t="s">
         <x:v>55</x:v>
@@ -8128,7 +8131,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="AB48" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AC48" s="12" t="s">
         <x:v>62</x:v>
@@ -8143,7 +8146,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AG48" s="12" t="s">
-        <x:v>139</x:v>
+        <x:v>142</x:v>
       </x:c>
       <x:c r="AH48" s="12" t="s">
         <x:v>49</x:v>
@@ -8155,10 +8158,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK48" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL48" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM48" s="12">
         <x:v>36</x:v>
@@ -8167,7 +8170,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AO48" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="AP48" s="12" t="s">
         <x:v>49</x:v>
@@ -8179,10 +8182,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS48" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT48" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU48" s="12">
         <x:v>36</x:v>
@@ -8215,7 +8218,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="BE48" s="12" t="s">
-        <x:v>65</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="BF48" s="12" t="s">
         <x:v>49</x:v>
@@ -8224,18 +8227,18 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="BH48" s="12" t="s">
-        <x:v>140</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="BI48" s="12">
         <x:v>285</x:v>
       </x:c>
       <x:c r="BJ48" s="12" t="s">
-        <x:v>141</x:v>
+        <x:v>143</x:v>
       </x:c>
     </x:row>
     <x:row r="49" spans="1:62">
       <x:c r="A49" s="11" t="s">
-        <x:v>142</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B49" s="12" t="s">
         <x:v>47</x:v>
@@ -8316,7 +8319,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="AB49" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AC49" s="12" t="s">
         <x:v>55</x:v>
@@ -8340,13 +8343,13 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="AJ49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AL49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM49" s="12">
         <x:v>37</x:v>
@@ -8364,19 +8367,19 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="AR49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT49" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU49" s="12">
         <x:v>37</x:v>
       </x:c>
       <x:c r="AV49" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AW49" s="12" t="s">
         <x:v>51</x:v>
@@ -8409,21 +8412,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG49" s="12">
-        <x:v>53</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="BH49" s="12" t="s">
-        <x:v>103</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="BI49" s="12">
-        <x:v>99</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="BJ49" s="12" t="s">
-        <x:v>101</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="50" spans="1:62">
       <x:c r="A50" s="11" t="s">
-        <x:v>143</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B50" s="12" t="s">
         <x:v>47</x:v>
@@ -8459,7 +8462,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="M50" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N50" s="12" t="s">
         <x:v>49</x:v>
@@ -8486,7 +8489,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="V50" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="W50" s="12">
         <x:v>38</x:v>
@@ -8528,13 +8531,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="AJ50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="AL50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM50" s="12">
         <x:v>38</x:v>
@@ -8552,13 +8555,13 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="AR50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AS50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT50" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU50" s="12">
         <x:v>38</x:v>
@@ -8597,24 +8600,24 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG50" s="12">
-        <x:v>45</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="BH50" s="12" t="s">
         <x:v>101</x:v>
       </x:c>
       <x:c r="BI50" s="12">
-        <x:v>63</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="BJ50" s="12" t="s">
-        <x:v>115</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="51" spans="1:62">
       <x:c r="A51" s="11" t="s">
-        <x:v>144</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B51" s="12" t="s">
-        <x:v>89</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C51" s="12">
         <x:v>39</x:v>
@@ -8719,10 +8722,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK51" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL51" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM51" s="12">
         <x:v>39</x:v>
@@ -8743,10 +8746,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS51" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT51" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU51" s="12">
         <x:v>39</x:v>
@@ -8788,13 +8791,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="BH51" s="12" t="s">
-        <x:v>145</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="BI51" s="12">
         <x:v>133</x:v>
       </x:c>
       <x:c r="BJ51" s="12" t="s">
-        <x:v>146</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="52" spans="1:62">
@@ -8802,7 +8805,7 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="B52" s="12" t="s">
-        <x:v>133</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="C52" s="12">
         <x:v>40</x:v>
@@ -8907,10 +8910,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK52" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL52" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM52" s="12">
         <x:v>40</x:v>
@@ -8931,10 +8934,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS52" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT52" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU52" s="12">
         <x:v>40</x:v>
@@ -8976,13 +8979,13 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH52" s="12" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BI52" s="12">
         <x:v>5</x:v>
       </x:c>
       <x:c r="BJ52" s="12" t="s">
-        <x:v>112</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="53" spans="1:62">
@@ -9050,7 +9053,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="V53" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="W53" s="12">
         <x:v>41</x:v>
@@ -9083,7 +9086,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="AG53" s="12" t="s">
-        <x:v>149</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="AH53" s="12" t="s">
         <x:v>49</x:v>
@@ -9092,13 +9095,13 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="AJ53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AK53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="AL53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM53" s="12">
         <x:v>41</x:v>
@@ -9116,13 +9119,13 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="AR53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AS53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="AT53" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU53" s="12">
         <x:v>41</x:v>
@@ -9161,21 +9164,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG53" s="12">
-        <x:v>88</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="BH53" s="12" t="s">
-        <x:v>150</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="BI53" s="12">
-        <x:v>114</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="BJ53" s="12" t="s">
-        <x:v>83</x:v>
+        <x:v>99</x:v>
       </x:c>
     </x:row>
     <x:row r="54" spans="1:62">
       <x:c r="A54" s="11" t="s">
-        <x:v>151</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B54" s="12" t="s">
         <x:v>47</x:v>
@@ -9280,13 +9283,13 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="AJ54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM54" s="12">
         <x:v>42</x:v>
@@ -9304,13 +9307,13 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="AR54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AS54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT54" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU54" s="12">
         <x:v>42</x:v>
@@ -9349,21 +9352,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG54" s="12">
-        <x:v>26</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="BH54" s="12" t="s">
-        <x:v>115</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BI54" s="12">
-        <x:v>73</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="BJ54" s="12" t="s">
-        <x:v>87</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="55" spans="1:62">
       <x:c r="A55" s="11" t="s">
-        <x:v>152</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="B55" s="12" t="s">
         <x:v>47</x:v>
@@ -9399,7 +9402,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="M55" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N55" s="12" t="s">
         <x:v>59</x:v>
@@ -9468,13 +9471,13 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="AJ55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AK55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM55" s="12">
         <x:v>43</x:v>
@@ -9492,19 +9495,19 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="AR55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AS55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT55" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU55" s="12">
         <x:v>43</x:v>
       </x:c>
       <x:c r="AV55" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AW55" s="12" t="s">
         <x:v>49</x:v>
@@ -9537,21 +9540,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG55" s="12">
-        <x:v>27</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="BH55" s="12" t="s">
-        <x:v>115</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="BI55" s="12">
-        <x:v>29</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="BJ55" s="12" t="s">
-        <x:v>106</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="56" spans="1:62">
       <x:c r="A56" s="11" t="s">
-        <x:v>153</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B56" s="12" t="s">
         <x:v>47</x:v>
@@ -9656,13 +9659,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="AJ56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AL56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM56" s="12">
         <x:v>44</x:v>
@@ -9680,13 +9683,13 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="AR56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="AT56" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU56" s="12">
         <x:v>44</x:v>
@@ -9725,21 +9728,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG56" s="12">
-        <x:v>71</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="BH56" s="12" t="s">
-        <x:v>71</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="BI56" s="12">
-        <x:v>77</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="BJ56" s="12" t="s">
-        <x:v>92</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="57" spans="1:62">
       <x:c r="A57" s="11" t="s">
-        <x:v>154</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B57" s="12" t="s">
         <x:v>47</x:v>
@@ -9844,13 +9847,13 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="AJ57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AL57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM57" s="12">
         <x:v>45</x:v>
@@ -9868,13 +9871,13 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="AR57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AT57" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU57" s="12">
         <x:v>45</x:v>
@@ -9895,7 +9898,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="BA57" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB57" s="12" t="s">
         <x:v>49</x:v>
@@ -9913,13 +9916,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG57" s="12">
-        <x:v>37</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="BH57" s="12" t="s">
-        <x:v>74</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="BI57" s="12">
-        <x:v>33</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="BJ57" s="12" t="s">
         <x:v>57</x:v>
@@ -9927,7 +9930,7 @@
     </x:row>
     <x:row r="58" spans="1:62">
       <x:c r="A58" s="11" t="s">
-        <x:v>155</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B58" s="12" t="s">
         <x:v>47</x:v>
@@ -9948,7 +9951,7 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="H58" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="I58" s="12" t="s">
         <x:v>48</x:v>
@@ -10023,7 +10026,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="AG58" s="12" t="s">
-        <x:v>70</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AH58" s="12" t="s">
         <x:v>49</x:v>
@@ -10032,13 +10035,13 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="AJ58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AK58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="AL58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM58" s="12">
         <x:v>46</x:v>
@@ -10056,13 +10059,13 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="AR58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="AS58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT58" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU58" s="12">
         <x:v>46</x:v>
@@ -10083,7 +10086,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="BA58" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB58" s="12" t="s">
         <x:v>49</x:v>
@@ -10101,21 +10104,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG58" s="12">
-        <x:v>63</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BH58" s="12" t="s">
-        <x:v>156</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="BI58" s="12">
-        <x:v>63</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BJ58" s="12" t="s">
-        <x:v>156</x:v>
+        <x:v>155</x:v>
       </x:c>
     </x:row>
     <x:row r="59" spans="1:62">
       <x:c r="A59" s="11" t="s">
-        <x:v>157</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B59" s="12" t="s">
         <x:v>47</x:v>
@@ -10220,13 +10223,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="AJ59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="AL59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM59" s="12">
         <x:v>47</x:v>
@@ -10244,13 +10247,13 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="AR59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="AT59" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU59" s="12">
         <x:v>47</x:v>
@@ -10271,7 +10274,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="BA59" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB59" s="12" t="s">
         <x:v>49</x:v>
@@ -10289,21 +10292,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG59" s="12">
-        <x:v>65</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BH59" s="12" t="s">
-        <x:v>134</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="BI59" s="12">
-        <x:v>65</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BJ59" s="12" t="s">
-        <x:v>134</x:v>
+        <x:v>155</x:v>
       </x:c>
     </x:row>
     <x:row r="60" spans="1:62">
       <x:c r="A60" s="11" t="s">
-        <x:v>158</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B60" s="12" t="s">
         <x:v>47</x:v>
@@ -10339,7 +10342,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="M60" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="N60" s="12" t="s">
         <x:v>49</x:v>
@@ -10408,13 +10411,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AJ60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="AK60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="AL60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM60" s="12">
         <x:v>48</x:v>
@@ -10432,13 +10435,13 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="AR60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="AS60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT60" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU60" s="12">
         <x:v>48</x:v>
@@ -10459,7 +10462,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="BA60" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BB60" s="12" t="s">
         <x:v>49</x:v>
@@ -10477,21 +10480,21 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BG60" s="12">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="BH60" s="12" t="s">
-        <x:v>57</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="BI60" s="12">
-        <x:v>15</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="BJ60" s="12" t="s">
-        <x:v>57</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="61" spans="1:62">
       <x:c r="A61" s="11" t="s">
-        <x:v>159</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B61" s="12" t="s">
         <x:v>47</x:v>
@@ -10599,10 +10602,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK61" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL61" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM61" s="12">
         <x:v>49</x:v>
@@ -10623,16 +10626,16 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS61" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT61" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU61" s="12">
         <x:v>49</x:v>
       </x:c>
       <x:c r="AV61" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AW61" s="12" t="s">
         <x:v>49</x:v>
@@ -10644,7 +10647,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="AZ61" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BA61" s="12" t="s">
         <x:v>49</x:v>
@@ -10656,7 +10659,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="BD61" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="BE61" s="12" t="s">
         <x:v>54</x:v>
@@ -10668,18 +10671,18 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="BH61" s="12" t="s">
-        <x:v>111</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="BI61" s="12">
         <x:v>6</x:v>
       </x:c>
       <x:c r="BJ61" s="12" t="s">
-        <x:v>111</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="62" spans="1:62">
       <x:c r="A62" s="11" t="s">
-        <x:v>160</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B62" s="12" t="s">
         <x:v>47</x:v>
@@ -10787,10 +10790,10 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AK62" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AL62" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AM62" s="12">
         <x:v>50</x:v>
@@ -10811,16 +10814,16 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="AS62" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AT62" s="12" t="s">
-        <x:v>53</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="AU62" s="12">
         <x:v>50</x:v>
       </x:c>
       <x:c r="AV62" s="12" t="s">
-        <x:v>64</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="AW62" s="12" t="s">
         <x:v>49</x:v>
@@ -10856,72 +10859,72 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="BH62" s="12" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="BI62" s="12">
         <x:v>0</x:v>
       </x:c>
       <x:c r="BJ62" s="12" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
     </x:row>
     <x:row r="63" spans="1:62">
       <x:c r="A63" s="13" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="B63" s="13" t="s">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="C63" s="7" t="s">
         <x:v>161</x:v>
-      </x:c>
-      <x:c r="B63" s="13" t="s">
-        <x:v>161</x:v>
-      </x:c>
-      <x:c r="C63" s="7" t="s">
-        <x:v>162</x:v>
       </x:c>
       <x:c r="D63" s="7"/>
       <x:c r="E63" s="7"/>
       <x:c r="F63" s="7"/>
       <x:c r="G63" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="H63" s="7"/>
       <x:c r="I63" s="7"/>
       <x:c r="J63" s="7"/>
       <x:c r="K63" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="L63" s="7"/>
       <x:c r="M63" s="7"/>
       <x:c r="N63" s="7"/>
       <x:c r="O63" s="7" t="s">
-        <x:v>164</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="P63" s="7"/>
       <x:c r="Q63" s="7"/>
       <x:c r="R63" s="7"/>
       <x:c r="S63" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="T63" s="7"/>
       <x:c r="U63" s="7"/>
       <x:c r="V63" s="7"/>
       <x:c r="W63" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="X63" s="7"/>
       <x:c r="Y63" s="7"/>
       <x:c r="Z63" s="7"/>
       <x:c r="AA63" s="7" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="AB63" s="7"/>
       <x:c r="AC63" s="7"/>
       <x:c r="AD63" s="7"/>
       <x:c r="AE63" s="7" t="s">
-        <x:v>166</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="AF63" s="7"/>
       <x:c r="AG63" s="7"/>
       <x:c r="AH63" s="7"/>
       <x:c r="AI63" s="7" t="s">
-        <x:v>164</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="AJ63" s="7"/>
       <x:c r="AK63" s="7"/>
@@ -10933,25 +10936,25 @@
       <x:c r="AO63" s="7"/>
       <x:c r="AP63" s="7"/>
       <x:c r="AQ63" s="7" t="s">
-        <x:v>164</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="AR63" s="7"/>
       <x:c r="AS63" s="7"/>
       <x:c r="AT63" s="7"/>
       <x:c r="AU63" s="7" t="s">
-        <x:v>165</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="AV63" s="7"/>
       <x:c r="AW63" s="7"/>
       <x:c r="AX63" s="7"/>
       <x:c r="AY63" s="7" t="s">
-        <x:v>168</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="AZ63" s="7"/>
       <x:c r="BA63" s="7"/>
       <x:c r="BB63" s="7"/>
       <x:c r="BC63" s="7" t="s">
-        <x:v>169</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="BD63" s="7"/>
       <x:c r="BE63" s="7"/>
@@ -10963,37 +10966,37 @@
     </x:row>
     <x:row r="65" spans="1:62">
       <x:c r="A65" s="14" t="s">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
     </x:row>
     <x:row r="66" spans="1:62">
       <x:c r="A66" s="13" t="s">
-        <x:v>171</x:v>
+        <x:v>172</x:v>
       </x:c>
     </x:row>
     <x:row r="67" spans="1:62">
       <x:c r="A67" s="13" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="68" spans="1:62">
       <x:c r="A68" s="13" t="s">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
     </x:row>
     <x:row r="69" spans="1:62">
       <x:c r="A69" s="13" t="s">
-        <x:v>174</x:v>
+        <x:v>175</x:v>
       </x:c>
     </x:row>
     <x:row r="70" spans="1:62">
       <x:c r="A70" s="13" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="71" spans="1:62">
       <x:c r="A71" s="13" t="s">
-        <x:v>176</x:v>
+        <x:v>177</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>